<commit_message>
fix bulk upload system
</commit_message>
<xml_diff>
--- a/trial 1(AutoRecovered) - Copy.xlsx
+++ b/trial 1(AutoRecovered) - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mohamed adel work\cesar-store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDA37AD-0074-46EB-857E-077856970B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112BEA7D-5E65-4399-8BDA-6F7D05829FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{791D22A4-40A8-4DDB-9123-A17DB6BCCBDF}"/>
   </bookViews>
@@ -1779,6 +1779,9 @@
       <c r="E2" s="5">
         <v>439.73124999999999</v>
       </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
       <c r="G2" t="s">
         <v>12</v>
       </c>
@@ -1809,6 +1812,9 @@
       <c r="E3" s="5">
         <v>238.71124999999998</v>
       </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
       <c r="G3" t="s">
         <v>12</v>
       </c>
@@ -1835,6 +1841,9 @@
       <c r="E4" s="5">
         <v>1587</v>
       </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
@@ -1861,6 +1870,9 @@
       <c r="E5" s="5">
         <v>1851.5</v>
       </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
       <c r="G5" t="s">
         <v>12</v>
       </c>
@@ -1887,6 +1899,9 @@
       <c r="E6" s="5">
         <v>1719.25</v>
       </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
       <c r="G6" t="s">
         <v>12</v>
       </c>
@@ -1913,6 +1928,9 @@
       <c r="E7" s="5">
         <v>1917.625</v>
       </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
       <c r="G7" t="s">
         <v>380</v>
       </c>
@@ -1939,6 +1957,9 @@
       <c r="E8" s="5">
         <v>168.61875000000001</v>
       </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
       <c r="G8" t="s">
         <v>380</v>
       </c>
@@ -1965,6 +1986,9 @@
       <c r="E9" s="5">
         <v>462.875</v>
       </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
       <c r="G9" t="s">
         <v>380</v>
       </c>
@@ -1991,6 +2015,9 @@
       <c r="E10" s="5">
         <v>74.721249999999998</v>
       </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
       <c r="G10" t="s">
         <v>380</v>
       </c>
@@ -2017,6 +2044,9 @@
       <c r="E11" s="5">
         <v>227.47000000000003</v>
       </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
       <c r="G11" t="s">
         <v>380</v>
       </c>
@@ -2043,6 +2073,9 @@
       <c r="E12" s="5">
         <v>156.61190474999998</v>
       </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
       <c r="G12" t="s">
         <v>380</v>
       </c>
@@ -2069,6 +2102,9 @@
       <c r="E13" s="5">
         <v>78.027499999999989</v>
       </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
       <c r="G13" t="s">
         <v>380</v>
       </c>
@@ -2095,6 +2131,9 @@
       <c r="E14" s="5">
         <v>271.11250000000001</v>
       </c>
+      <c r="F14">
+        <v>4</v>
+      </c>
       <c r="G14" t="s">
         <v>380</v>
       </c>
@@ -2121,6 +2160,9 @@
       <c r="E15" s="5">
         <v>133.41009700000001</v>
       </c>
+      <c r="F15">
+        <v>4</v>
+      </c>
       <c r="G15" t="s">
         <v>380</v>
       </c>
@@ -2147,6 +2189,9 @@
       <c r="E16" s="5">
         <v>101.8325</v>
       </c>
+      <c r="F16">
+        <v>4</v>
+      </c>
       <c r="G16" t="s">
         <v>380</v>
       </c>
@@ -2173,6 +2218,9 @@
       <c r="E17" s="5">
         <v>101.8325</v>
       </c>
+      <c r="F17">
+        <v>4</v>
+      </c>
       <c r="G17" t="s">
         <v>380</v>
       </c>
@@ -2199,6 +2247,9 @@
       <c r="E18" s="5">
         <v>101.8325</v>
       </c>
+      <c r="F18">
+        <v>4</v>
+      </c>
       <c r="G18" t="s">
         <v>376</v>
       </c>
@@ -2225,6 +2276,9 @@
       <c r="E19" s="5">
         <v>101.8325</v>
       </c>
+      <c r="F19">
+        <v>4</v>
+      </c>
       <c r="G19" t="s">
         <v>376</v>
       </c>
@@ -2251,6 +2305,9 @@
       <c r="E20" s="5">
         <v>101.8325</v>
       </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
       <c r="G20" t="s">
         <v>376</v>
       </c>
@@ -2277,6 +2334,9 @@
       <c r="E21" s="5">
         <v>39.674999999999997</v>
       </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
       <c r="G21" t="s">
         <v>376</v>
       </c>
@@ -2303,6 +2363,9 @@
       <c r="E22" s="5">
         <v>417.63161374999999</v>
       </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
       <c r="G22" t="s">
         <v>376</v>
       </c>
@@ -2329,6 +2392,9 @@
       <c r="E23" s="5">
         <v>481.43641974999997</v>
       </c>
+      <c r="F23">
+        <v>4</v>
+      </c>
       <c r="G23" t="s">
         <v>376</v>
       </c>
@@ -2355,6 +2421,9 @@
       <c r="E24" s="5">
         <v>276.40249999999997</v>
       </c>
+      <c r="F24">
+        <v>4</v>
+      </c>
       <c r="G24" t="s">
         <v>376</v>
       </c>
@@ -2381,6 +2450,9 @@
       <c r="E25" s="5">
         <v>116.0097</v>
       </c>
+      <c r="F25">
+        <v>4</v>
+      </c>
       <c r="G25" t="s">
         <v>376</v>
       </c>
@@ -2407,6 +2479,9 @@
       <c r="E26" s="5">
         <v>75.405643749999996</v>
       </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
       <c r="G26" t="s">
         <v>376</v>
       </c>
@@ -2433,6 +2508,9 @@
       <c r="E27" s="5">
         <v>101.8325</v>
       </c>
+      <c r="F27">
+        <v>4</v>
+      </c>
       <c r="G27" t="s">
         <v>376</v>
       </c>
@@ -2459,6 +2537,9 @@
       <c r="E28" s="5">
         <v>251.27500000000001</v>
       </c>
+      <c r="F28">
+        <v>4</v>
+      </c>
       <c r="G28" t="s">
         <v>376</v>
       </c>
@@ -2485,6 +2566,9 @@
       <c r="E29" s="5">
         <v>296.24</v>
       </c>
+      <c r="F29">
+        <v>4</v>
+      </c>
       <c r="G29" t="s">
         <v>377</v>
       </c>
@@ -2511,6 +2595,9 @@
       <c r="E30" s="5">
         <v>1653.125</v>
       </c>
+      <c r="F30">
+        <v>4</v>
+      </c>
       <c r="G30" t="s">
         <v>377</v>
       </c>
@@ -2537,6 +2624,9 @@
       <c r="E31" s="5">
         <v>395.75812500000001</v>
       </c>
+      <c r="F31">
+        <v>4</v>
+      </c>
       <c r="G31" t="s">
         <v>377</v>
       </c>
@@ -2563,6 +2653,9 @@
       <c r="E32" s="5">
         <v>207.301875</v>
       </c>
+      <c r="F32">
+        <v>4</v>
+      </c>
       <c r="G32" t="s">
         <v>377</v>
       </c>
@@ -2589,6 +2682,9 @@
       <c r="E33" s="5">
         <v>121.80925925</v>
       </c>
+      <c r="F33">
+        <v>4</v>
+      </c>
       <c r="G33" t="s">
         <v>377</v>
       </c>
@@ -2615,6 +2711,9 @@
       <c r="E34" s="5">
         <v>110.29650000000001</v>
       </c>
+      <c r="F34">
+        <v>4</v>
+      </c>
       <c r="G34" t="s">
         <v>377</v>
       </c>
@@ -2641,6 +2740,9 @@
       <c r="E35" s="5">
         <v>232.00617500000001</v>
       </c>
+      <c r="F35">
+        <v>4</v>
+      </c>
       <c r="G35" t="s">
         <v>377</v>
       </c>
@@ -2667,6 +2769,9 @@
       <c r="E36" s="5">
         <v>382.82896825000006</v>
       </c>
+      <c r="F36">
+        <v>4</v>
+      </c>
       <c r="G36" t="s">
         <v>377</v>
       </c>
@@ -2693,6 +2798,9 @@
       <c r="E37" s="5">
         <v>276.40249999999997</v>
       </c>
+      <c r="F37">
+        <v>4</v>
+      </c>
       <c r="G37" t="s">
         <v>377</v>
       </c>
@@ -2719,6 +2827,9 @@
       <c r="E38" s="5">
         <v>238.71124999999998</v>
       </c>
+      <c r="F38">
+        <v>4</v>
+      </c>
       <c r="G38" t="s">
         <v>378</v>
       </c>
@@ -2745,6 +2856,9 @@
       <c r="E39" s="5">
         <v>185.15</v>
       </c>
+      <c r="F39">
+        <v>4</v>
+      </c>
       <c r="G39" t="s">
         <v>378</v>
       </c>
@@ -2771,6 +2885,9 @@
       <c r="E40" s="5">
         <v>188.45625000000001</v>
       </c>
+      <c r="F40">
+        <v>4</v>
+      </c>
       <c r="G40" t="s">
         <v>378</v>
       </c>
@@ -2797,6 +2914,9 @@
       <c r="E41" s="5">
         <v>188.45625000000001</v>
       </c>
+      <c r="F41">
+        <v>4</v>
+      </c>
       <c r="G41" t="s">
         <v>378</v>
       </c>
@@ -2823,6 +2943,9 @@
       <c r="E42" s="5">
         <v>188.45625000000001</v>
       </c>
+      <c r="F42">
+        <v>4</v>
+      </c>
       <c r="G42" t="s">
         <v>378</v>
       </c>
@@ -2849,6 +2972,9 @@
       <c r="E43" s="5">
         <v>188.45625000000001</v>
       </c>
+      <c r="F43">
+        <v>4</v>
+      </c>
       <c r="G43" t="s">
         <v>378</v>
       </c>
@@ -2875,6 +3001,9 @@
       <c r="E44" s="5">
         <v>188.45625000000001</v>
       </c>
+      <c r="F44">
+        <v>4</v>
+      </c>
       <c r="G44" t="s">
         <v>378</v>
       </c>
@@ -2901,6 +3030,9 @@
       <c r="E45" s="5">
         <v>188.45625000000001</v>
       </c>
+      <c r="F45">
+        <v>4</v>
+      </c>
       <c r="G45" t="s">
         <v>378</v>
       </c>
@@ -2927,6 +3059,9 @@
       <c r="E46" s="5">
         <v>396.75</v>
       </c>
+      <c r="F46">
+        <v>4</v>
+      </c>
       <c r="G46" t="s">
         <v>378</v>
       </c>
@@ -2953,6 +3088,9 @@
       <c r="E47" s="5">
         <v>244.66249999999999</v>
       </c>
+      <c r="F47">
+        <v>4</v>
+      </c>
       <c r="G47" t="s">
         <v>379</v>
       </c>
@@ -2979,6 +3117,9 @@
       <c r="E48" s="5">
         <v>244.66249999999999</v>
       </c>
+      <c r="F48">
+        <v>4</v>
+      </c>
       <c r="G48" t="s">
         <v>379</v>
       </c>
@@ -3005,6 +3146,9 @@
       <c r="E49" s="5">
         <v>238.05</v>
       </c>
+      <c r="F49">
+        <v>4</v>
+      </c>
       <c r="G49" t="s">
         <v>379</v>
       </c>
@@ -3031,6 +3175,9 @@
       <c r="E50" s="5">
         <v>158.69999999999999</v>
       </c>
+      <c r="F50">
+        <v>4</v>
+      </c>
       <c r="G50" t="s">
         <v>379</v>
       </c>
@@ -3057,6 +3204,9 @@
       <c r="E51" s="5">
         <v>152.08750000000001</v>
       </c>
+      <c r="F51">
+        <v>4</v>
+      </c>
       <c r="G51" t="s">
         <v>379</v>
       </c>
@@ -3083,6 +3233,9 @@
       <c r="E52" s="5">
         <v>112.41249999999999</v>
       </c>
+      <c r="F52">
+        <v>4</v>
+      </c>
       <c r="G52" t="s">
         <v>379</v>
       </c>
@@ -3109,6 +3262,9 @@
       <c r="E53" s="5">
         <v>218.21250000000001</v>
       </c>
+      <c r="F53">
+        <v>4</v>
+      </c>
       <c r="G53" t="s">
         <v>379</v>
       </c>
@@ -3135,6 +3291,9 @@
       <c r="E54" s="5">
         <v>92.575000000000003</v>
       </c>
+      <c r="F54">
+        <v>4</v>
+      </c>
       <c r="G54" t="s">
         <v>379</v>
       </c>
@@ -3161,6 +3320,9 @@
       <c r="E55" s="5">
         <v>59.512500000000003</v>
       </c>
+      <c r="F55">
+        <v>4</v>
+      </c>
       <c r="G55" t="s">
         <v>380</v>
       </c>
@@ -3187,6 +3349,9 @@
       <c r="E56" s="5">
         <v>145.47499999999999</v>
       </c>
+      <c r="F56">
+        <v>4</v>
+      </c>
       <c r="G56" t="s">
         <v>380</v>
       </c>
@@ -3213,6 +3378,9 @@
       <c r="E57" s="5">
         <v>317.39999999999998</v>
       </c>
+      <c r="F57">
+        <v>4</v>
+      </c>
       <c r="G57" t="s">
         <v>380</v>
       </c>
@@ -3239,6 +3407,9 @@
       <c r="E58" s="5">
         <v>482.71249999999998</v>
       </c>
+      <c r="F58">
+        <v>4</v>
+      </c>
       <c r="G58" t="s">
         <v>380</v>
       </c>
@@ -3265,6 +3436,9 @@
       <c r="E59" s="5">
         <v>462.875</v>
       </c>
+      <c r="F59">
+        <v>4</v>
+      </c>
       <c r="G59" t="s">
         <v>380</v>
       </c>
@@ -3290,6 +3464,9 @@
       </c>
       <c r="E60" s="5">
         <v>296.24</v>
+      </c>
+      <c r="F60">
+        <v>4</v>
       </c>
       <c r="G60" t="s">
         <v>380</v>

</xml_diff>